<commit_message>
Add SMRT9999 to master price list
</commit_message>
<xml_diff>
--- a/master_price_list.xlsx
+++ b/master_price_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I178"/>
+  <dimension ref="A1:I179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5497,6 +5497,35 @@
       <c r="G178" t="n">
         <v>8906187980543</v>
       </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>179</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>SMRT9999</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>999</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>95030020</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>SMRT9999</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>